<commit_message>
simulation: created simulation for 12V igntion
Having problems with bleed through on the FET during startup. It's small, but not ideal for a pyrotechnic initiator. May abandon this design.
</commit_message>
<xml_diff>
--- a/4_BOM/12V_MR-Launch-Controller_BOM.xlsx
+++ b/4_BOM/12V_MR-Launch-Controller_BOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\MR-Launch-Controller\4_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5ED99D42-0F01-4A7E-93EE-740810560C27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C574B1FE-C42A-4F2A-A800-7815B04EBDAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="My Lists Worksheet" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="106">
   <si>
     <t>Index</t>
   </si>
@@ -169,42 +169,9 @@
     <t>$0.30</t>
   </si>
   <si>
-    <t>Keystone Electronics</t>
-  </si>
-  <si>
-    <t>BATTERY HOLDER AA 4 CELL PC PIN</t>
-  </si>
-  <si>
-    <t>36-2477-ND</t>
-  </si>
-  <si>
-    <t>1.87000</t>
-  </si>
-  <si>
-    <t>$1.87</t>
-  </si>
-  <si>
-    <t>BT1</t>
-  </si>
-  <si>
-    <t>ZTX718</t>
-  </si>
-  <si>
-    <t>Diodes Incorporated</t>
-  </si>
-  <si>
-    <t>TRANS PNP 20V 2.5A E-LINE</t>
-  </si>
-  <si>
-    <t>ZTX718-ND</t>
-  </si>
-  <si>
     <t>0.77000</t>
   </si>
   <si>
-    <t>$1.54</t>
-  </si>
-  <si>
     <t>ANT11SF1CQE</t>
   </si>
   <si>
@@ -229,9 +196,6 @@
     <t>YAGEO</t>
   </si>
   <si>
-    <t>P6KE, DO-204AC, 6.4V, 11.3V, BOX</t>
-  </si>
-  <si>
     <t>0.38000</t>
   </si>
   <si>
@@ -274,21 +238,6 @@
     <t>R2, R3, R6</t>
   </si>
   <si>
-    <t>0ZRG0250FF1E</t>
-  </si>
-  <si>
-    <t>PTC RESET FUSE 30V 2.5A RADIAL</t>
-  </si>
-  <si>
-    <t>5923-0ZRG0250FF1E-ND</t>
-  </si>
-  <si>
-    <t>P6KE7.5A/B</t>
-  </si>
-  <si>
-    <t>13-P6KE7.5A/B-ND</t>
-  </si>
-  <si>
     <t>Q1</t>
   </si>
   <si>
@@ -359,6 +308,36 @@
   </si>
   <si>
     <t>CF14JT62R0CT-ND</t>
+  </si>
+  <si>
+    <t>P6KE18A</t>
+  </si>
+  <si>
+    <t>TVS DIODE 15.3VWM 25.2V DO204AC</t>
+  </si>
+  <si>
+    <t>P6KE18ALFCT-ND</t>
+  </si>
+  <si>
+    <t>0ZRS1000FF1A</t>
+  </si>
+  <si>
+    <t>PTC RESET FUSE 32V 10A RADIAL</t>
+  </si>
+  <si>
+    <t>5923-0ZRS1000FF1A-ND</t>
+  </si>
+  <si>
+    <t>2N3906</t>
+  </si>
+  <si>
+    <t>Diotec Semiconductor</t>
+  </si>
+  <si>
+    <t>TRANS PNP 40V 0.2A TO-92</t>
+  </si>
+  <si>
+    <t>4878-2N3906CT-ND</t>
   </si>
 </sst>
 </file>
@@ -707,7 +686,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q16"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="23" customWidth="1"/>
@@ -787,10 +766,10 @@
         <v>1729128</v>
       </c>
       <c r="C2" t="s">
-        <v>101</v>
+        <v>84</v>
       </c>
       <c r="D2" t="s">
-        <v>102</v>
+        <v>85</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -802,7 +781,7 @@
         <v>33</v>
       </c>
       <c r="I2" t="s">
-        <v>103</v>
+        <v>86</v>
       </c>
       <c r="J2">
         <v>0.95</v>
@@ -964,7 +943,7 @@
         <v>1</v>
       </c>
       <c r="M5" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="N5" t="s">
         <v>19</v>
@@ -1014,7 +993,7 @@
         <v>1</v>
       </c>
       <c r="M6" t="s">
-        <v>97</v>
+        <v>80</v>
       </c>
       <c r="N6" t="s">
         <v>19</v>
@@ -1031,16 +1010,16 @@
     </row>
     <row r="7" spans="1:17">
       <c r="A7">
-        <v>6</v>
-      </c>
-      <c r="B7">
-        <v>2477</v>
+        <v>7</v>
+      </c>
+      <c r="B7" t="s">
+        <v>102</v>
       </c>
       <c r="C7" t="s">
-        <v>49</v>
+        <v>103</v>
       </c>
       <c r="D7" t="s">
-        <v>50</v>
+        <v>104</v>
       </c>
       <c r="F7">
         <v>1</v>
@@ -1052,19 +1031,19 @@
         <v>33</v>
       </c>
       <c r="I7" t="s">
-        <v>51</v>
+        <v>105</v>
       </c>
       <c r="J7" t="s">
-        <v>52</v>
-      </c>
-      <c r="K7" t="s">
-        <v>53</v>
+        <v>49</v>
+      </c>
+      <c r="K7">
+        <v>0.14000000000000001</v>
       </c>
       <c r="L7">
         <v>1</v>
       </c>
       <c r="M7" t="s">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="N7" t="s">
         <v>19</v>
@@ -1076,21 +1055,21 @@
         <v>21</v>
       </c>
       <c r="Q7" t="s">
-        <v>51</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:17">
       <c r="A8">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="C8" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="D8" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -1102,19 +1081,19 @@
         <v>33</v>
       </c>
       <c r="I8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="J8" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="K8" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="L8">
         <v>1</v>
       </c>
       <c r="M8" t="s">
-        <v>89</v>
+        <v>56</v>
       </c>
       <c r="N8" t="s">
         <v>19</v>
@@ -1123,48 +1102,48 @@
         <v>20</v>
       </c>
       <c r="P8" t="s">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="Q8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:17">
       <c r="A9">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>96</v>
       </c>
       <c r="C9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="D9" t="s">
-        <v>63</v>
+        <v>97</v>
       </c>
       <c r="F9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H9" t="s">
-        <v>33</v>
+        <v>17</v>
       </c>
       <c r="I9" t="s">
-        <v>64</v>
+        <v>98</v>
       </c>
       <c r="J9" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="K9" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="L9">
         <v>1</v>
       </c>
       <c r="M9" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="N9" t="s">
         <v>19</v>
@@ -1173,48 +1152,48 @@
         <v>20</v>
       </c>
       <c r="P9" t="s">
-        <v>36</v>
+        <v>21</v>
       </c>
       <c r="Q9" t="s">
-        <v>64</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:17">
       <c r="A10">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B10" t="s">
-        <v>87</v>
+        <v>99</v>
       </c>
       <c r="C10" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="D10" t="s">
-        <v>69</v>
+        <v>100</v>
       </c>
       <c r="F10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H10" t="s">
-        <v>17</v>
+        <v>45</v>
       </c>
       <c r="I10" t="s">
-        <v>88</v>
-      </c>
-      <c r="J10" t="s">
-        <v>70</v>
-      </c>
-      <c r="K10" t="s">
-        <v>71</v>
+        <v>101</v>
+      </c>
+      <c r="J10">
+        <v>2.2400000000000002</v>
+      </c>
+      <c r="K10">
+        <v>2.2400000000000002</v>
       </c>
       <c r="L10">
         <v>1</v>
       </c>
       <c r="M10" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
       <c r="N10" t="s">
         <v>19</v>
@@ -1226,45 +1205,45 @@
         <v>21</v>
       </c>
       <c r="Q10" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
     </row>
     <row r="11" spans="1:17">
       <c r="A11">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>84</v>
+        <v>63</v>
       </c>
       <c r="C11" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="D11" t="s">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="F11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G11">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H11" t="s">
         <v>45</v>
       </c>
       <c r="I11" t="s">
-        <v>86</v>
-      </c>
-      <c r="J11">
-        <v>0.57999999999999996</v>
-      </c>
-      <c r="K11">
-        <v>0.57999999999999996</v>
+        <v>66</v>
+      </c>
+      <c r="J11" t="s">
+        <v>67</v>
+      </c>
+      <c r="K11" t="s">
+        <v>48</v>
       </c>
       <c r="L11">
         <v>1</v>
       </c>
       <c r="M11" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="N11" t="s">
         <v>19</v>
@@ -1276,21 +1255,21 @@
         <v>21</v>
       </c>
       <c r="Q11" t="s">
-        <v>86</v>
+        <v>66</v>
       </c>
     </row>
     <row r="12" spans="1:17">
       <c r="A12">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>75</v>
+        <v>68</v>
       </c>
       <c r="C12" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="D12" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="F12">
         <v>3</v>
@@ -1302,10 +1281,10 @@
         <v>45</v>
       </c>
       <c r="I12" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="J12" t="s">
-        <v>79</v>
+        <v>67</v>
       </c>
       <c r="K12" t="s">
         <v>48</v>
@@ -1314,7 +1293,7 @@
         <v>1</v>
       </c>
       <c r="M12" t="s">
-        <v>98</v>
+        <v>71</v>
       </c>
       <c r="N12" t="s">
         <v>19</v>
@@ -1326,71 +1305,65 @@
         <v>21</v>
       </c>
       <c r="Q12" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:17">
       <c r="A13">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B13" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="C13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" t="s">
         <v>76</v>
       </c>
-      <c r="D13" t="s">
-        <v>81</v>
-      </c>
       <c r="F13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G13">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H13" t="s">
         <v>45</v>
       </c>
       <c r="I13" t="s">
-        <v>82</v>
-      </c>
-      <c r="J13" t="s">
-        <v>79</v>
-      </c>
-      <c r="K13" t="s">
-        <v>48</v>
+        <v>77</v>
+      </c>
+      <c r="J13">
+        <v>1.1200000000000001</v>
+      </c>
+      <c r="K13">
+        <v>1.1200000000000001</v>
       </c>
       <c r="L13">
         <v>1</v>
       </c>
       <c r="M13" t="s">
-        <v>83</v>
-      </c>
-      <c r="N13" t="s">
-        <v>19</v>
+        <v>73</v>
       </c>
       <c r="O13" t="s">
         <v>20</v>
       </c>
-      <c r="P13" t="s">
-        <v>21</v>
-      </c>
       <c r="Q13" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:17">
       <c r="A14">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B14" t="s">
+        <v>90</v>
+      </c>
+      <c r="C14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" t="s">
         <v>91</v>
-      </c>
-      <c r="C14" t="s">
-        <v>92</v>
-      </c>
-      <c r="D14" t="s">
-        <v>93</v>
       </c>
       <c r="F14">
         <v>1</v>
@@ -1402,39 +1375,39 @@
         <v>45</v>
       </c>
       <c r="I14" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="J14">
-        <v>1.1200000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="K14">
-        <v>1.1200000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="L14">
         <v>1</v>
       </c>
       <c r="M14" t="s">
-        <v>90</v>
+        <v>78</v>
       </c>
       <c r="O14" t="s">
         <v>20</v>
       </c>
       <c r="Q14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:17">
       <c r="A15">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B15" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
       <c r="C15" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="D15" t="s">
-        <v>108</v>
+        <v>89</v>
       </c>
       <c r="F15">
         <v>1</v>
@@ -1446,7 +1419,7 @@
         <v>45</v>
       </c>
       <c r="I15" t="s">
-        <v>109</v>
+        <v>88</v>
       </c>
       <c r="J15">
         <v>0.1</v>
@@ -1458,27 +1431,27 @@
         <v>1</v>
       </c>
       <c r="M15" t="s">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="O15" t="s">
         <v>20</v>
       </c>
       <c r="Q15" t="s">
-        <v>107</v>
+        <v>87</v>
       </c>
     </row>
     <row r="16" spans="1:17">
       <c r="A16">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B16" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="C16" t="s">
-        <v>76</v>
+        <v>64</v>
       </c>
       <c r="D16" t="s">
-        <v>106</v>
+        <v>94</v>
       </c>
       <c r="F16">
         <v>1</v>
@@ -1490,7 +1463,7 @@
         <v>45</v>
       </c>
       <c r="I16" t="s">
-        <v>105</v>
+        <v>95</v>
       </c>
       <c r="J16">
         <v>0.1</v>
@@ -1502,57 +1475,13 @@
         <v>1</v>
       </c>
       <c r="M16" t="s">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="O16" t="s">
         <v>20</v>
       </c>
       <c r="Q16" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17" t="s">
-        <v>110</v>
-      </c>
-      <c r="C17" t="s">
-        <v>76</v>
-      </c>
-      <c r="D17" t="s">
-        <v>111</v>
-      </c>
-      <c r="F17">
-        <v>1</v>
-      </c>
-      <c r="G17">
-        <v>1</v>
-      </c>
-      <c r="H17" t="s">
-        <v>45</v>
-      </c>
-      <c r="I17" t="s">
-        <v>112</v>
-      </c>
-      <c r="J17">
-        <v>0.1</v>
-      </c>
-      <c r="K17">
-        <v>0.1</v>
-      </c>
-      <c r="L17">
-        <v>1</v>
-      </c>
-      <c r="M17" t="s">
-        <v>100</v>
-      </c>
-      <c r="O17" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q17" t="s">
-        <v>110</v>
+        <v>93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>